<commit_message>
D5: título de la matriz a ERS v2.0
</commit_message>
<xml_diff>
--- a/04_Trazabilidad/matriz_e2e.xlsx
+++ b/04_Trazabilidad/matriz_e2e.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="464">
   <si>
-    <t xml:space="preserve">MATRIZ DE TRAZABILIDAD EXTREMO A EXTREMO — ERS SIMPA v1.1</t>
+    <t xml:space="preserve">MATRIZ DE TRAZABILIDAD EXTREMO A EXTREMO — ERS SIMPA v2.0</t>
   </si>
   <si>
     <t xml:space="preserve">Cadena completa: Fuente → Requisito → Caso de uso → Clase/Módulo → Proceso DFD → Estado → Criterio BDD → Caso de prueba. Hacia atrás: columnas B y C. Hacia adelante: columnas G a M. La columna N declara el estado de la traza de cada fila.</t>
@@ -1762,7 +1762,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1778,7 +1778,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1786,7 +1786,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6118,15 +6118,15 @@
   <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="s">
         <v>445</v>
       </c>
@@ -6141,7 +6141,7 @@
       <c r="E2" s="31"/>
       <c r="F2" s="31"/>
     </row>
-    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
         <v>7</v>
       </c>
@@ -6641,22 +6641,22 @@
         <v>456</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="36" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>463</v>
       </c>

</xml_diff>